<commit_message>
Docs: las observaciones del revisor se atribuyen al cliente (SEVENS)
Se quita el nombre del revisor técnico de los entregables y de docs/flujos.md
por pedido del equipo; sus observaciones figuran como del cliente.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PtGmXDVgEBa1Hp6paBTjbG
</commit_message>
<xml_diff>
--- a/entregables/SIGRO - Product Backlog v6.xlsx
+++ b/entregables/SIGRO - Product Backlog v6.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>v6 · 15/10/2026 · incorpora los acuerdos de la reunión con el cliente y la revisión del Ing. Junior Cercado</t>
+          <t>v6 · 15/10/2026 · incorpora los acuerdos de la reunión con el cliente y la revisión técnica del cliente</t>
         </is>
       </c>
     </row>
@@ -6469,7 +6469,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Reunión con SEVENS INGENIEROS SAC (oct. 2026) · revisión del Ing. Junior Cercado (15/10/2026)</t>
+          <t>Reunión con SEVENS INGENIEROS SAC (oct. 2026) · revisión técnica del cliente (15/10/2026)</t>
         </is>
       </c>
     </row>
@@ -6640,7 +6640,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Tanto el cliente como el Ing. Junior Cercado coinciden en que exigen cruzar partidas y metrados, con alto esfuerzo y poco retorno para este alcance.</t>
+          <t>El cliente coincide en que exigen cruzar partidas y metrados, con alto esfuerzo y poco retorno para este alcance.</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -6662,7 +6662,7 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>El Ing. Junior Cercado recomendó mover a Post-MVP lo de bajo valor frente al problema central.</t>
+          <t>El cliente recomendó mover a Post-MVP lo de bajo valor frente al problema central.</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">

</xml_diff>